<commit_message>
feat: implement POS seed generation and validation
</commit_message>
<xml_diff>
--- a/data/raw/promotions/promociones_2026-41.xlsx
+++ b/data/raw/promotions/promociones_2026-41.xlsx
@@ -484,7 +484,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>MA-HOG-0001</t>
+          <t>SKU-ARTANDCRA-CO-01019</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -505,12 +505,12 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>MA-BEL-0002</t>
+          <t>SKU-ART-CO-00691</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>CANAL_ECOMMERCE</t>
+          <t>CO_E-commerce Propio</t>
         </is>
       </c>
       <c r="C3" t="n">
@@ -526,12 +526,12 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>MA-TEC-0003</t>
+          <t>SKU-AGRINDAND-CO-00556</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>CANAL_MARKETPLACE</t>
+          <t>CO_Marketplace Propietario</t>
         </is>
       </c>
       <c r="C4" t="n">
@@ -547,7 +547,7 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>MA-DEP-0004</t>
+          <t>SKU-AUD-CO-00309</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
@@ -568,7 +568,7 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>MA-REL-0005</t>
+          <t>SKU-AGRINDAND-PE-00560</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
@@ -589,7 +589,7 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>MA-MUE-0006</t>
+          <t>SKU-AIRCON-EC-00367</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
@@ -610,7 +610,7 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>MA-COC-0007</t>
+          <t>SKU-AGRINDAND-BO-00558</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
@@ -631,7 +631,7 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>MA-JAR-0008</t>
+          <t>SKU-AGRINDAND-CL-00559</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
@@ -652,7 +652,7 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>MA-ANI-0009</t>
+          <t>SKU-BEDBATTAB-CO-00048</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
@@ -673,12 +673,12 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>MA-TOY-0010</t>
+          <t>SKU-AIRCON-PE-00365</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>CANAL_ECOMMERCE</t>
+          <t>PE_E-commerce Propio</t>
         </is>
       </c>
       <c r="C11" t="n">

</xml_diff>